<commit_message>
Daily NSE scan: 2026-08-24
</commit_message>
<xml_diff>
--- a/output/2026-08-24/enriched_analysis.xlsx
+++ b/output/2026-08-24/enriched_analysis.xlsx
@@ -616,7 +616,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Gandhar Oil Refinery (India) Limited</t>
+          <t>GANDHAR OIL REFINERY (INDIA) LIMITED</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -1290,27 +1290,27 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>SIGIND</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PNGS Reva Diamond Jewellery Limited</t>
+          <t>Signet Industries Limited</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Buy on Breakout</t>
+          <t>Strong Buy Setup</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F9" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G9" t="n">
         <v>20</v>
@@ -1319,82 +1319,84 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>547.45</v>
+        <v>67.88</v>
       </c>
       <c r="J9" t="n">
-        <v>390.61</v>
+        <v>70.27</v>
       </c>
       <c r="K9" t="n">
-        <v>40.2</v>
+        <v>-3.4</v>
       </c>
       <c r="L9" t="n">
-        <v>63.09</v>
+        <v>72.56999999999999</v>
       </c>
       <c r="M9" t="n">
-        <v>8.02</v>
+        <v>0.7</v>
       </c>
       <c r="N9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>21-08-2026</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>0.467</v>
+        <v>0.347</v>
       </c>
       <c r="Q9" t="n">
-        <v>1716</v>
+        <v>202</v>
       </c>
       <c r="R9" t="n">
-        <v>20.3</v>
+        <v>8.58</v>
       </c>
       <c r="S9" t="n">
-        <v>581</v>
+        <v>17</v>
       </c>
       <c r="T9" t="n">
-        <v>34</v>
+        <v>27.97</v>
       </c>
       <c r="U9" t="n">
-        <v>881</v>
+        <v>17</v>
       </c>
       <c r="V9" t="n">
-        <v>8.58</v>
+        <v>2.73</v>
       </c>
       <c r="W9" t="n">
-        <v>22</v>
+        <v>13.7</v>
       </c>
       <c r="X9" t="n">
-        <v>0.33</v>
+        <v>1.86</v>
       </c>
       <c r="Y9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z9" t="n">
-        <v>29</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="AA9" t="n">
-        <v>450.64</v>
-      </c>
-      <c r="AB9" t="inlineStr"/>
+        <v>53.82</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>51.03</v>
+      </c>
       <c r="AC9" t="n">
-        <v>31.4</v>
+        <v>41.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SIGIND</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Signet Industries Limited</t>
+          <t>PNGS Reva Diamond Jewellery Limited</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1405,7 +1407,7 @@
         <v>20</v>
       </c>
       <c r="F10" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G10" t="n">
         <v>20</v>
@@ -1414,69 +1416,67 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>67.88</v>
+        <v>547.45</v>
       </c>
       <c r="J10" t="n">
-        <v>68.84999999999999</v>
+        <v>390.61</v>
       </c>
       <c r="K10" t="n">
-        <v>-1.4</v>
+        <v>40.2</v>
       </c>
       <c r="L10" t="n">
-        <v>72.56999999999999</v>
+        <v>63.09</v>
       </c>
       <c r="M10" t="n">
-        <v>0.46</v>
+        <v>8.02</v>
       </c>
       <c r="N10" t="n">
         <v>3</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>19-08-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>0.228</v>
+        <v>0.467</v>
       </c>
       <c r="Q10" t="n">
-        <v>202</v>
+        <v>1716</v>
       </c>
       <c r="R10" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="S10" t="n">
+        <v>581</v>
+      </c>
+      <c r="T10" t="n">
+        <v>34</v>
+      </c>
+      <c r="U10" t="n">
+        <v>881</v>
+      </c>
+      <c r="V10" t="n">
         <v>8.58</v>
       </c>
-      <c r="S10" t="n">
-        <v>17</v>
-      </c>
-      <c r="T10" t="n">
-        <v>27.97</v>
-      </c>
-      <c r="U10" t="n">
-        <v>17</v>
-      </c>
-      <c r="V10" t="n">
-        <v>2.73</v>
-      </c>
       <c r="W10" t="n">
-        <v>13.7</v>
+        <v>22</v>
       </c>
       <c r="X10" t="n">
-        <v>1.86</v>
+        <v>0.33</v>
       </c>
       <c r="Y10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z10" t="n">
-        <v>9.140000000000001</v>
+        <v>29</v>
       </c>
       <c r="AA10" t="n">
-        <v>53.82</v>
-      </c>
-      <c r="AB10" t="n">
-        <v>51.03</v>
-      </c>
+        <v>450.64</v>
+      </c>
+      <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="n">
-        <v>41.3</v>
+        <v>31.4</v>
       </c>
     </row>
     <row r="11">
@@ -1679,7 +1679,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>INE577L01016</t>
+          <t>STEL HOLDINGS LIMITED</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -3318,7 +3318,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Ganesh Consumer Products Limited</t>
+          <t>GANESH CONSUMER PRODUCTS LIMITED</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -3979,7 +3979,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>OBCL LIMITED</t>
+          <t>OBCL LIMITED (FORMERLY KNOWN AS ORISSA BENGAL CARRIER LIMITED)</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -5017,7 +5017,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Gandhar Oil Refinery (India) Limited</t>
+          <t>GANDHAR OIL REFINERY (INDIA) LIMITED</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -5257,70 +5257,70 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PNGSREVA</t>
+          <t>SIGIND</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PNGS Reva Diamond Jewellery Limited</t>
+          <t>Signet Industries Limited</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>547.45</v>
+        <v>67.88</v>
       </c>
       <c r="D9" t="n">
-        <v>390.61</v>
+        <v>70.27</v>
       </c>
       <c r="E9" t="n">
-        <v>40.2</v>
+        <v>-3.4</v>
       </c>
       <c r="F9" t="n">
-        <v>63.09</v>
+        <v>72.56999999999999</v>
       </c>
       <c r="G9" t="n">
-        <v>8.02</v>
+        <v>0.7</v>
       </c>
       <c r="H9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>21-08-2026</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SIGIND</t>
+          <t>PNGSREVA</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Signet Industries Limited</t>
+          <t>PNGS Reva Diamond Jewellery Limited</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>67.88</v>
+        <v>547.45</v>
       </c>
       <c r="D10" t="n">
-        <v>68.84999999999999</v>
+        <v>390.61</v>
       </c>
       <c r="E10" t="n">
-        <v>-1.4</v>
+        <v>40.2</v>
       </c>
       <c r="F10" t="n">
-        <v>72.56999999999999</v>
+        <v>63.09</v>
       </c>
       <c r="G10" t="n">
-        <v>0.46</v>
+        <v>8.02</v>
       </c>
       <c r="H10" t="n">
         <v>3</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>19-08-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
     </row>
@@ -5402,7 +5402,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>INE577L01016</t>
+          <t>STEL HOLDINGS LIMITED</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -5997,7 +5997,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Ganesh Consumer Products Limited</t>
+          <t>GANESH CONSUMER PRODUCTS LIMITED</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -6242,7 +6242,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>OBCL LIMITED</t>
+          <t>OBCL LIMITED (FORMERLY KNOWN AS ORISSA BENGAL CARRIER LIMITED)</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -6677,7 +6677,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9">
@@ -6697,7 +6697,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">

</xml_diff>